<commit_message>
Das Datum zurAbbuchung bzw Überweisung soll noch in die Rechnung geschriebne werden. eine Rechnungsübersicht soll noch erzeugt werden (Einnahmen, Ausgaben, Mitgliedsbeitrag).
</commit_message>
<xml_diff>
--- a/data/Mitgliederliste-Reidlinger.xlsx
+++ b/data/Mitgliederliste-Reidlinger.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" codeName="DieseArbeitsmappe" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14364" windowHeight="6468"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22044" windowHeight="8712"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="54">
   <si>
     <t>Name</t>
   </si>
@@ -163,12 +163,33 @@
   </si>
   <si>
     <t>Rabatt-Cent</t>
+  </si>
+  <si>
+    <t>Mandatsreferenz</t>
+  </si>
+  <si>
+    <t>MandatsDatum</t>
+  </si>
+  <si>
+    <t>R003</t>
+  </si>
+  <si>
+    <t>R005</t>
+  </si>
+  <si>
+    <t>R006</t>
+  </si>
+  <si>
+    <t>M</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -239,7 +260,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -261,14 +282,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="12">
     <dxf>
       <font>
         <strike val="0"/>
@@ -307,6 +335,13 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -352,8 +387,8 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="WJ1" pivot="0" count="2">
-      <tableStyleElement type="wholeTable" dxfId="9"/>
-      <tableStyleElement type="headerRow" dxfId="8"/>
+      <tableStyleElement type="wholeTable" dxfId="11"/>
+      <tableStyleElement type="headerRow" dxfId="10"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -368,14 +403,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabelle3" displayName="Tabelle3" ref="A3:O13" totalsRowShown="0">
-  <autoFilter ref="A3:O13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabelle3" displayName="Tabelle3" ref="A3:Q14" totalsRowShown="0">
+  <autoFilter ref="A3:Q14"/>
   <sortState ref="A2:M4">
     <sortCondition ref="A1:A4"/>
   </sortState>
-  <tableColumns count="15">
-    <tableColumn id="1" name="lfd. Nummer" dataDxfId="7"/>
-    <tableColumn id="2" name="Folgezeile" dataDxfId="6"/>
+  <tableColumns count="17">
+    <tableColumn id="1" name="lfd. Nummer" dataDxfId="9"/>
+    <tableColumn id="2" name="Folgezeile" dataDxfId="8"/>
+    <tableColumn id="17" name="Mandatsreferenz" dataDxfId="7"/>
+    <tableColumn id="16" name="MandatsDatum" dataDxfId="6"/>
     <tableColumn id="14" name="Anrede"/>
     <tableColumn id="3" name="Name"/>
     <tableColumn id="4" name="Vorname"/>
@@ -658,135 +695,151 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="13.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" style="7" customWidth="1"/>
-    <col min="4" max="4" width="12.77734375" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" customWidth="1"/>
-    <col min="6" max="6" width="22.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="12.21875" style="8" customWidth="1"/>
-    <col min="9" max="9" width="27.44140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="20.109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="24.44140625" customWidth="1"/>
-    <col min="12" max="12" width="43.5546875" customWidth="1"/>
-    <col min="13" max="13" width="11.77734375" style="9" customWidth="1"/>
-    <col min="14" max="14" width="43.21875" style="4" customWidth="1"/>
-    <col min="15" max="15" width="15.21875" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.21875" style="14" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" style="7" customWidth="1"/>
+    <col min="6" max="6" width="12.77734375" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" customWidth="1"/>
+    <col min="8" max="8" width="22.77734375" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="12.21875" style="8" customWidth="1"/>
+    <col min="11" max="11" width="27.44140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="20.109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="24.44140625" customWidth="1"/>
+    <col min="14" max="14" width="43.5546875" customWidth="1"/>
+    <col min="15" max="15" width="11.77734375" style="9" customWidth="1"/>
+    <col min="16" max="16" width="43.21875" style="4" customWidth="1"/>
+    <col min="17" max="17" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="B1" s="13" t="s">
+    <row r="1" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+      <c r="B1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>0</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>1</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>2</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="J3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
         <v>7</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="N3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="O3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="P3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="O3" t="s">
+      <c r="Q3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="14">
+        <v>45742</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>9</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>21</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="J4" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K4" t="s">
+      <c r="M4" t="s">
         <v>13</v>
       </c>
-      <c r="L4" s="4" t="s">
+      <c r="N4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1.1000000000000001</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="I5" s="3"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="9">
+      <c r="E5" s="2"/>
+      <c r="K5" s="3"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="9">
         <v>100</v>
       </c>
-      <c r="N5" s="4" t="s">
+      <c r="P5" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>1.2</v>
       </c>
@@ -794,19 +847,21 @@
         <v>29</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="1"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="4" t="s">
+      <c r="D6" s="14"/>
+      <c r="E6" s="2"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="1"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="O6" s="12">
+      <c r="Q6" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>1.3</v>
       </c>
@@ -814,19 +869,21 @@
         <v>29</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="1"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="4" t="s">
+      <c r="D7" s="14"/>
+      <c r="E7" s="2"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="1"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="9"/>
+      <c r="P7" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="O7" s="12">
+      <c r="Q7" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>1.4</v>
       </c>
@@ -834,164 +891,200 @@
         <v>29</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="1"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="4" t="s">
+      <c r="D8" s="14"/>
+      <c r="E8" s="2"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="1"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="O8" s="12">
+      <c r="Q8" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
+    <row r="9" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="17">
+        <v>46143</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="2"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="1"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="P9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q9" s="12"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
         <v>2</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="E10" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D9" t="s">
+      <c r="F10" t="s">
         <v>8</v>
       </c>
-      <c r="E9" t="s">
+      <c r="G10" t="s">
         <v>19</v>
       </c>
-      <c r="F9" t="s">
+      <c r="H10" t="s">
         <v>22</v>
       </c>
-      <c r="G9" t="s">
+      <c r="I10" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="J10" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="K10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="L10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K9" t="s">
+      <c r="M10" t="s">
         <v>13</v>
       </c>
-      <c r="L9" s="4" t="s">
+      <c r="N10" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
         <v>3</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="14">
+        <v>45658</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D10" t="s">
+      <c r="F11" t="s">
         <v>35</v>
       </c>
-      <c r="E10" t="s">
+      <c r="G11" t="s">
         <v>45</v>
       </c>
-      <c r="F10" t="s">
+      <c r="H11" t="s">
         <v>24</v>
       </c>
-      <c r="G10" t="s">
+      <c r="I11" t="s">
         <v>10</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="J11" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="K11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="L11" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="K10" t="s">
+      <c r="M11" t="s">
         <v>37</v>
       </c>
-      <c r="L10" s="4" t="s">
+      <c r="N11" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="N10" s="6"/>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
+      <c r="P11" s="6"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A12" s="2">
         <v>3.1</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="I11" s="3"/>
-      <c r="L11" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
-        <v>3.2</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="I12" s="3"/>
-      <c r="L12" s="4" t="s">
+      <c r="E12" s="2"/>
+      <c r="K12" s="3"/>
+      <c r="N12" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A13" s="2">
+        <v>3.2</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K13" s="3"/>
+      <c r="N13" s="4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A13" s="2">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
         <v>4</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C14" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" s="14">
+        <v>45689</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D13" t="s">
+      <c r="F14" t="s">
         <v>38</v>
       </c>
-      <c r="E13" t="s">
+      <c r="G14" t="s">
         <v>39</v>
       </c>
-      <c r="F13" t="s">
+      <c r="H14" t="s">
         <v>40</v>
       </c>
-      <c r="G13" t="s">
+      <c r="I14" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="8" t="s">
+      <c r="J14" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="K14" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="L14" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="K13" t="s">
+      <c r="M14" t="s">
         <v>43</v>
       </c>
-      <c r="L13" s="4" t="s">
+      <c r="N14" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="N14" s="5"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="L15" s="11"/>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="P15" s="5"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="N16" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B1:I1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="I9" r:id="rId1"/>
-    <hyperlink ref="I4" r:id="rId2"/>
-    <hyperlink ref="I10" r:id="rId3"/>
-    <hyperlink ref="I13" r:id="rId4"/>
+    <hyperlink ref="K10" r:id="rId1"/>
+    <hyperlink ref="K4" r:id="rId2"/>
+    <hyperlink ref="K11" r:id="rId3"/>
+    <hyperlink ref="K14" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId5"/>

</xml_diff>